<commit_message>
Assigment1 part 1 exercise 1
</commit_message>
<xml_diff>
--- a/Assigment1.xlsx
+++ b/Assigment1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jinCh\Documents\ProjectManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{28847E6F-E3D7-4AA1-9062-A434A9C2C48C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B27E5716-E5FD-4D65-BA0F-D4E5B2E61374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{112DB047-7552-42C9-9ED2-8F2AE23E1317}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="FeasibilityStudy" sheetId="1" r:id="rId1"/>
     <sheet name="ReferenceData" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">FeasibilityStudy!$C$5:$D$9</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>Year</t>
   </si>
@@ -76,6 +79,114 @@
   </si>
   <si>
     <t>Alternative Investment Rate</t>
+  </si>
+  <si>
+    <t>* Cost (Year 0): "Initial capital expenditure required for project launch"</t>
+  </si>
+  <si>
+    <t>* Income: "Revenue generated by the system. Values are assumed to be distributed uniformly throughout each month"</t>
+  </si>
+  <si>
+    <t>* Net Cash Flow: "Total annual liquidity calculated as Income minus Costs"</t>
+  </si>
+  <si>
+    <t>* Cumulative Cash Flow: "The running total of net cash flows, used to identify the break-even point"</t>
+  </si>
+  <si>
+    <t>Exercise 1</t>
+  </si>
+  <si>
+    <t>a) Break Even Point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          The project breaks even, as we can see, during Year 3, as that is when the Cumulative Cash Flow turns positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Net Cash Flow during Year 3: 1300,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Remaining to recover ar start of Year 3: 300,00 €</t>
+  </si>
+  <si>
+    <t>b) Return on Investment (ROI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          The ROI measures the total efficiency of the project over 4 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Total Net Benefit: Sum of all NCF = 2300,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Total Costs: 500 + 800 + 1000 + 1000 + 1000 = 4300,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Manual Calculation: ROI = (2300/4300) * 100 = 53,49%</t>
+  </si>
+  <si>
+    <t>c) 50% Performance in Year 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          If Year 1 income drops to 50% (from 1000 € to 500 €)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - New NCF Year 1: 500 - 800 = -300,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - New Cumulative CF Year 1: -500 - 300 = -800,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - New Cumulative CF Year 2: -800 + 0 = -800,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - New Cumulative CF Year 3: -800 + 1300 = +500,00 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          The project still breaks even in Year 3, but a bit later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Time Calculation: 800/1300 = 0,6154 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Time Calculation: 300/1300 = 0,2307 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Months: 0,2307 * 12 months = 2,769 months --&gt; 2 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Days: 0,769 * 22 working days = 16,92 days --&gt; 17 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Months: 0,6154 * 12 = 7,38 months --&gt; 7 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Days: 0,38 * 22 = 8,36 days --&gt; 8,4 days</t>
+  </si>
+  <si>
+    <t>The adjusted BET is 2 years, 7 months and 8,4 days</t>
+  </si>
+  <si>
+    <t>d) NPV and IRR (for scenario c)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          Using the discounted rate K = 5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - Flows: -500, -300, 0, +1300, +1300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - NPV Calculations:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                    NPV = -500 + (-300/1,05^1) + (0/1,05^2) + (1300/1,05^3) + (1300/1,05^4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                    NPV = -500 - 285,71 + 0 + 1122,99 + 1069,51 = 1406,79 €</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - IRR: Solving for r when NPV = 0, you get approximately 28,32%</t>
+  </si>
+  <si>
+    <t>Since the IRR (28,32%) is significantly higher than the return on alternative investments (10%), the project is interesting and profitable</t>
   </si>
 </sst>
 </file>
@@ -83,9 +194,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +230,20 @@
       <sz val="10"/>
       <color rgb="FF434343"/>
       <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="36"/>
+      <color theme="1"/>
+      <name val="Amasis MT Pro Medium"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -237,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -266,11 +391,21 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -606,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF2A8C3-C4F3-44C3-B42C-C9B988A89C62}">
-  <dimension ref="B1:F7"/>
+  <dimension ref="B1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.5546875" customWidth="1"/>
@@ -614,100 +749,492 @@
     <col min="3" max="6" width="22.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:6" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+    </row>
+    <row r="3" spans="2:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="11">
-        <f>C3-D3</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="11">
-        <f>E3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="2:6" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="4">
-        <v>1</v>
-      </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="11">
-        <f t="shared" ref="E4:E7" si="0">C4-D4</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="11">
-        <f>F3+E4</f>
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
-        <v>2</v>
-      </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
+        <v>0</v>
+      </c>
+      <c r="C5" s="10">
+        <v>500</v>
+      </c>
+      <c r="D5" s="10">
+        <v>0</v>
+      </c>
       <c r="E5" s="11">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>D5-C5</f>
+        <v>-500</v>
       </c>
       <c r="F5" s="11">
-        <f t="shared" ref="F5:F7" si="1">F4+E5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <f>E5</f>
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="4">
-        <v>3</v>
-      </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
+        <v>1</v>
+      </c>
+      <c r="C6" s="10">
+        <v>800</v>
+      </c>
+      <c r="D6" s="10">
+        <v>1000</v>
+      </c>
       <c r="E6" s="11">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" ref="E6:E9" si="0">D6-C6</f>
+        <v>200</v>
       </c>
       <c r="F6" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>F5+E6</f>
+        <v>-300</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3">
-        <v>4</v>
-      </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
+        <v>2</v>
+      </c>
+      <c r="C7" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D7" s="10">
+        <v>1000</v>
+      </c>
       <c r="E7" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F7" s="11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+        <f>F6+E7</f>
+        <v>-300</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="4">
+        <v>3</v>
+      </c>
+      <c r="C8" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D8" s="10">
+        <v>2300</v>
+      </c>
+      <c r="E8" s="11">
+        <f t="shared" si="0"/>
+        <v>1300</v>
+      </c>
+      <c r="F8" s="11">
+        <f>F7+E8</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="3">
+        <v>4</v>
+      </c>
+      <c r="C9" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D9" s="10">
+        <v>2300</v>
+      </c>
+      <c r="E9" s="11">
+        <f t="shared" si="0"/>
+        <v>1300</v>
+      </c>
+      <c r="F9" s="11">
+        <f>F8+E9</f>
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B31" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B32" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+    </row>
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B33" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B34" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="13"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B35" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B36" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B38" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="13"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B39" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B40" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B41" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B43" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="13"/>
+    </row>
+    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B45" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13"/>
+      <c r="F45" s="13"/>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B46" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B47" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="13"/>
+      <c r="F47" s="13"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B48" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B49" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B50" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B51" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="13"/>
+      <c r="F51" s="13"/>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B53" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="H56" s="12"/>
     </row>
   </sheetData>
+  <mergeCells count="36">
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B21:F21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B51:F51"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a positive numeric value (e.g., 1234,56)" sqref="C5:D9" xr:uid="{D0791DB1-D684-4D7E-A456-DA8AC201638A}">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed a mistake in the section d
</commit_message>
<xml_diff>
--- a/Assigment1.xlsx
+++ b/Assigment1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jinCh\Documents\ProjectManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B27E5716-E5FD-4D65-BA0F-D4E5B2E61374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E4FEBF-1604-40FD-A7C8-3CCC47865FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{112DB047-7552-42C9-9ED2-8F2AE23E1317}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
   <si>
     <t>Year</t>
   </si>
@@ -183,10 +183,13 @@
     <t xml:space="preserve">                    NPV = -500 - 285,71 + 0 + 1122,99 + 1069,51 = 1406,79 €</t>
   </si>
   <si>
-    <t xml:space="preserve">          - IRR: Solving for r when NPV = 0, you get approximately 28,32%</t>
-  </si>
-  <si>
     <t>Since the IRR (28,32%) is significantly higher than the return on alternative investments (10%), the project is interesting and profitable</t>
+  </si>
+  <si>
+    <t>**Calculated whith the excel formula**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          - IRR: Solving for r when NPV = 0, you get approximately 45,89%</t>
   </si>
 </sst>
 </file>
@@ -362,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -402,10 +405,22 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CF2A8C3-C4F3-44C3-B42C-C9B988A89C62}">
-  <dimension ref="B1:H56"/>
+  <dimension ref="B1:H64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.5546875" customWidth="1"/>
@@ -751,13 +766,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="2:6" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -873,331 +888,505 @@
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="14" t="s">
+      <c r="B13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="13"/>
-      <c r="F20" s="13"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="13" t="s">
+      <c r="B26" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="13" t="s">
+      <c r="B27" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="13" t="s">
+      <c r="B28" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="13" t="s">
-        <v>28</v>
-      </c>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+    </row>
+    <row r="32" spans="2:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B33" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="13"/>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B34" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B35" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C35" s="13"/>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="13"/>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B36" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B38" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C38" s="13"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
+    <row r="33" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="3">
+        <v>0</v>
+      </c>
+      <c r="C34" s="10">
+        <v>500</v>
+      </c>
+      <c r="D34" s="10">
+        <v>0</v>
+      </c>
+      <c r="E34" s="11">
+        <f>D34-C34</f>
+        <v>-500</v>
+      </c>
+      <c r="F34" s="11">
+        <f>E34</f>
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="4">
+        <v>1</v>
+      </c>
+      <c r="C35" s="10">
+        <v>800</v>
+      </c>
+      <c r="D35" s="10">
+        <v>500</v>
+      </c>
+      <c r="E35" s="11">
+        <f t="shared" ref="E35:E38" si="1">D35-C35</f>
+        <v>-300</v>
+      </c>
+      <c r="F35" s="11">
+        <f>F34+E35</f>
+        <v>-800</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="3">
+        <v>2</v>
+      </c>
+      <c r="C36" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D36" s="10">
+        <v>1000</v>
+      </c>
+      <c r="E36" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="F36" s="11">
+        <f>F35+E36</f>
+        <v>-800</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="4">
+        <v>3</v>
+      </c>
+      <c r="C37" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D37" s="10">
+        <v>2300</v>
+      </c>
+      <c r="E37" s="11">
+        <f t="shared" si="1"/>
+        <v>1300</v>
+      </c>
+      <c r="F37" s="11">
+        <f>F36+E37</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="3">
+        <v>4</v>
+      </c>
+      <c r="C38" s="10">
+        <v>1000</v>
+      </c>
+      <c r="D38" s="10">
+        <v>2300</v>
+      </c>
+      <c r="E38" s="11">
+        <f t="shared" si="1"/>
+        <v>1300</v>
+      </c>
+      <c r="F38" s="11">
+        <f>F37+E38</f>
+        <v>1800</v>
+      </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B39" s="13" t="s">
-        <v>34</v>
-      </c>
+      <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
       <c r="E39" s="13"/>
       <c r="F39" s="13"/>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B40" s="13" t="s">
+      <c r="B40" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B41" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+    </row>
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B42" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+    </row>
+    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B43" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+    </row>
+    <row r="44" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B44" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+    </row>
+    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B46" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="14"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+    </row>
+    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B47" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+    </row>
+    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B48" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="13"/>
-      <c r="D40" s="13"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-    </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B41" s="13" t="s">
+      <c r="C48" s="14"/>
+      <c r="D48" s="14"/>
+      <c r="E48" s="14"/>
+      <c r="F48" s="14"/>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B49" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C41" s="13"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-    </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B43" s="13" t="s">
+      <c r="C49" s="14"/>
+      <c r="D49" s="14"/>
+      <c r="E49" s="14"/>
+      <c r="F49" s="14"/>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B51" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="13"/>
-    </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B45" s="13" t="s">
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B53" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="13"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13"/>
-    </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B46" s="13" t="s">
+      <c r="C53" s="14"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="14"/>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B54" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-    </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B47" s="13" t="s">
+      <c r="C54" s="14"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="14"/>
+      <c r="F54" s="14"/>
+    </row>
+    <row r="55" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B55" s="13"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+    </row>
+    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B56" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C47" s="13"/>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13"/>
-    </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B48" s="13" t="s">
+      <c r="C56" s="14"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="14"/>
+      <c r="G56" s="13"/>
+    </row>
+    <row r="57" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B57" s="13"/>
+      <c r="C57" s="13"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+    </row>
+    <row r="58" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B58" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-    </row>
-    <row r="49" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B49" s="13" t="s">
+      <c r="C58" s="14"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="14"/>
+      <c r="F58" s="14"/>
+    </row>
+    <row r="59" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B59" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C49" s="13"/>
-      <c r="D49" s="13"/>
-      <c r="E49" s="13"/>
-      <c r="F49" s="13"/>
-    </row>
-    <row r="50" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B50" s="13" t="s">
+      <c r="C59" s="14"/>
+      <c r="D59" s="14"/>
+      <c r="E59" s="14"/>
+      <c r="F59" s="14"/>
+    </row>
+    <row r="60" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B60" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C50" s="13"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13"/>
-    </row>
-    <row r="51" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B51" s="13" t="s">
+      <c r="C60" s="14"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="14"/>
+      <c r="H60" s="12"/>
+    </row>
+    <row r="61" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B61" s="13"/>
+      <c r="C61" s="13"/>
+      <c r="D61" s="13"/>
+      <c r="E61" s="13"/>
+      <c r="F61" s="13"/>
+      <c r="H61" s="12"/>
+    </row>
+    <row r="62" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B62" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C62" s="14"/>
+      <c r="D62" s="14"/>
+      <c r="E62" s="14"/>
+      <c r="F62" s="14"/>
+    </row>
+    <row r="63" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B63" s="18" t="str">
+        <f>"IRR = "&amp;IRR(E34:E38)</f>
+        <v>IRR = 0,458902575504396</v>
+      </c>
+      <c r="C63" s="18"/>
+      <c r="D63" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E63" s="17"/>
+    </row>
+    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B64" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C51" s="13"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
-    </row>
-    <row r="53" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B53" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="C53" s="13"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="13"/>
-    </row>
-    <row r="56" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="H56" s="12"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="18"/>
+      <c r="F64" s="18"/>
+      <c r="G64" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B2:F2"/>
+  <mergeCells count="37">
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B54:F54"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="B59:F59"/>
+    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="B62:F62"/>
+    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B41:F41"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B51:F51"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B17:F17"/>
@@ -1210,28 +1399,14 @@
     <mergeCell ref="B26:F26"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="B43:F43"/>
-    <mergeCell ref="B53:G53"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B47:F47"/>
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B2:F2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a positive numeric value (e.g., 1234,56)" sqref="C5:D9" xr:uid="{D0791DB1-D684-4D7E-A456-DA8AC201638A}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a positive numeric value (e.g., 1234,56)" sqref="C5:D9 C34:D38" xr:uid="{D0791DB1-D684-4D7E-A456-DA8AC201638A}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>